<commit_message>
Checkpoint corrected corpus outputs for clean reproduction
</commit_message>
<xml_diff>
--- a/vignettes/vignette-1/distribution_stats.xlsx
+++ b/vignettes/vignette-1/distribution_stats.xlsx
@@ -465,16 +465,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C2" t="n">
         <v>376</v>
       </c>
       <c r="D2" t="n">
-        <v>0.024576</v>
+        <v>0.02454</v>
       </c>
       <c r="E2" t="n">
-        <v>0.135997</v>
+        <v>0.135901</v>
       </c>
       <c r="F2" t="n">
         <v>0.061784</v>
@@ -493,16 +493,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C3" t="n">
         <v>376</v>
       </c>
       <c r="D3" t="n">
-        <v>0.014633</v>
+        <v>0.014611</v>
       </c>
       <c r="E3" t="n">
-        <v>0.07030699999999999</v>
+        <v>0.070258</v>
       </c>
       <c r="F3" t="n">
         <v>0.04982</v>
@@ -523,10 +523,10 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>-0.009943</v>
+        <v>-0.009929</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.06569</v>
+        <v>-0.06564300000000001</v>
       </c>
       <c r="F4" t="n">
         <v>-0.011964</v>

</xml_diff>